<commit_message>
feat: Num Engineers config row, Type column fallback, optional management capacity
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/input_example_realistic_messy.xlsx
+++ b/data/examples/input_example_realistic_messy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/irina.migallon/dev/cli/planzen/data/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB573E7E-B0C9-D240-B72F-F13ECD8E661B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46F70AD-EEB7-0740-BE92-746D2729C098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="17300" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="680" windowWidth="17300" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="89">
   <si>
     <t>Estimation</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>Uniform</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Gaps</t>
   </si>
   <si>
     <t>Overhead</t>
@@ -818,12 +824,12 @@
   <cols>
     <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" customWidth="1"/>
-    <col min="4" max="4" width="13.5" customWidth="1"/>
+    <col min="10" max="10" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
@@ -831,9 +837,6 @@
       <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" t="s">
-        <v>10</v>
-      </c>
       <c r="E1" t="s">
         <v>1</v>
       </c>
@@ -843,100 +846,103 @@
       <c r="G1" t="s">
         <v>2</v>
       </c>
+      <c r="J1" t="s">
+        <v>10</v>
+      </c>
       <c r="K1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="Z1" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AA1" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AB1" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AC1" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="AD1" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="AE1" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AF1" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AG1" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AH1" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="AI1" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="AJ1" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="AK1" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AL1" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AM1" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="AN1" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AO1" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -973,16 +979,15 @@
     <row r="3" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="J3" s="4"/>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
@@ -1075,16 +1080,15 @@
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
+      <c r="J4" s="4"/>
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
       <c r="M4" s="8"/>
@@ -1167,16 +1171,15 @@
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="20"/>
       <c r="B5" s="20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
       <c r="E5" s="21"/>
       <c r="F5" s="21"/>
       <c r="G5" s="21"/>
       <c r="H5" s="21"/>
       <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
+      <c r="J5" s="20"/>
       <c r="K5" s="21"/>
       <c r="L5" s="21"/>
       <c r="M5" s="21"/>
@@ -1269,10 +1272,9 @@
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="20"/>
       <c r="B6" s="20" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
       <c r="E6" s="21"/>
       <c r="F6" s="21">
         <v>0.45</v>
@@ -1280,7 +1282,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
       <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
+      <c r="J6" s="20"/>
       <c r="K6" s="21"/>
       <c r="L6" s="21"/>
       <c r="M6" s="21"/>
@@ -1318,19 +1320,18 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="J7" s="4"/>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
@@ -1422,19 +1423,18 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
+      <c r="J8" s="4"/>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
@@ -1485,13 +1485,12 @@
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="J9" s="4"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
@@ -1531,13 +1530,12 @@
       <c r="A11" s="20"/>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
       <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
+      <c r="J11" s="20"/>
       <c r="K11" s="21"/>
       <c r="L11" s="21"/>
       <c r="M11" s="21"/>
@@ -1575,15 +1573,12 @@
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C12" s="4"/>
-      <c r="D12" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E12" s="8">
         <v>0</v>
       </c>
@@ -1594,7 +1589,9 @@
         <v>1.2</v>
       </c>
       <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="J12" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="K12" s="8">
         <v>1.9</v>
       </c>
@@ -1603,7 +1600,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
@@ -1660,9 +1657,6 @@
         <v>3</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E13" s="8">
         <v>0</v>
       </c>
@@ -1673,7 +1667,9 @@
         <v>1.2</v>
       </c>
       <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="J13" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="K13" s="8">
         <v>1.2</v>
       </c>
@@ -1682,7 +1678,7 @@
         <v>1.6</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O13" s="4">
         <v>0.1</v>
@@ -1770,12 +1766,9 @@
         <v>3</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C14" s="9"/>
-      <c r="D14" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E14" s="11">
         <v>0</v>
       </c>
@@ -1786,7 +1779,9 @@
         <v>1.2</v>
       </c>
       <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
+      <c r="J14" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="K14" s="11">
         <v>7.8</v>
       </c>
@@ -1795,7 +1790,7 @@
         <v>7.7</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O14" s="4">
         <v>0.6</v>
@@ -1887,13 +1882,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E15" s="8">
         <v>0</v>
@@ -1905,7 +1897,9 @@
         <v>1.2</v>
       </c>
       <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
+      <c r="J15" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="K15" s="8">
         <v>0.8</v>
       </c>
@@ -1914,7 +1908,7 @@
         <v>4.2</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="O15" s="4">
         <v>0</v>
@@ -1999,15 +1993,12 @@
     </row>
     <row r="16" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>14</v>
-      </c>
       <c r="C16" s="2"/>
-      <c r="D16" s="4">
-        <v>0</v>
-      </c>
       <c r="E16" s="8">
         <v>1</v>
       </c>
@@ -2018,9 +2009,11 @@
         <v>1.2</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="J16" s="8"/>
+        <v>27</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K16" s="8">
         <v>0</v>
       </c>
@@ -2029,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
@@ -2067,13 +2060,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="4">
-        <v>2.5</v>
+        <v>19</v>
       </c>
       <c r="E17" s="8">
         <v>1</v>
@@ -2085,7 +2075,9 @@
         <v>1.2</v>
       </c>
       <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
+      <c r="J17" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K17" s="8">
         <v>2.5</v>
       </c>
@@ -2094,7 +2086,7 @@
         <v>4.3</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
@@ -2171,9 +2163,6 @@
         <v>3</v>
       </c>
       <c r="C18" s="2"/>
-      <c r="D18" s="4">
-        <v>3</v>
-      </c>
       <c r="E18" s="8">
         <v>0</v>
       </c>
@@ -2184,7 +2173,9 @@
         <v>1.2</v>
       </c>
       <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="J18" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="K18" s="8">
         <v>0.1</v>
       </c>
@@ -2193,7 +2184,7 @@
         <v>2</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O18" s="4">
         <v>0</v>
@@ -2254,7 +2245,6 @@
         <v>3</v>
       </c>
       <c r="C19" s="2"/>
-      <c r="D19" s="4"/>
       <c r="E19" s="8">
         <v>0</v>
       </c>
@@ -2265,14 +2255,16 @@
         <v>1.2</v>
       </c>
       <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+      <c r="J19" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
       <c r="M19" s="15">
         <v>1</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
@@ -2322,13 +2314,10 @@
         <v>3</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="4">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="E20" s="8">
         <v>0</v>
@@ -2340,7 +2329,9 @@
         <v>1.2</v>
       </c>
       <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="J20" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K20" s="8">
         <v>1</v>
       </c>
@@ -2349,7 +2340,7 @@
         <v>1.2</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="O20" s="4"/>
       <c r="P20" s="4">
@@ -2410,13 +2401,12 @@
     </row>
     <row r="21" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C21" s="2"/>
-      <c r="D21" s="4"/>
       <c r="E21" s="8">
         <v>1</v>
       </c>
@@ -2427,7 +2417,9 @@
         <v>1.2</v>
       </c>
       <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="J21" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K21" s="8">
         <v>0</v>
       </c>
@@ -2436,7 +2428,7 @@
         <v>0.5</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
@@ -2476,10 +2468,9 @@
         <v>3</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2"/>
-      <c r="D22" s="4"/>
       <c r="E22" s="8">
         <v>0</v>
       </c>
@@ -2490,7 +2481,9 @@
         <v>1.2</v>
       </c>
       <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
+      <c r="J22" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K22" s="13">
         <v>0.4</v>
       </c>
@@ -2499,7 +2492,7 @@
         <v>0.6</v>
       </c>
       <c r="N22" s="16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
@@ -2545,14 +2538,11 @@
         <v>5</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="4">
-        <v>1</v>
-      </c>
       <c r="E23" s="8">
         <v>2</v>
       </c>
@@ -2563,14 +2553,16 @@
         <v>1.2</v>
       </c>
       <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="J23" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="K23" s="8">
         <v>0.6</v>
       </c>
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="17" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O23" s="4"/>
       <c r="P23" s="4">
@@ -2622,14 +2614,11 @@
         <v>5</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="4">
-        <v>0</v>
-      </c>
       <c r="E24" s="8">
         <v>2</v>
       </c>
@@ -2640,14 +2629,16 @@
         <v>1.2</v>
       </c>
       <c r="I24" s="4"/>
-      <c r="J24" s="8"/>
+      <c r="J24" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="K24" s="8">
         <v>2.4</v>
       </c>
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
@@ -2697,14 +2688,11 @@
         <v>5</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="4">
-        <v>0</v>
-      </c>
       <c r="E25" s="8">
         <v>2</v>
       </c>
@@ -2715,14 +2703,16 @@
         <v>1.2</v>
       </c>
       <c r="I25" s="4"/>
-      <c r="J25" s="8"/>
+      <c r="J25" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="K25" s="8">
         <v>1.9</v>
       </c>
       <c r="L25" s="8"/>
       <c r="M25" s="8"/>
       <c r="N25" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
@@ -2770,12 +2760,11 @@
         <v>5</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="4"/>
       <c r="E26" s="8">
         <v>4</v>
       </c>
@@ -2784,14 +2773,16 @@
         <v>1.3</v>
       </c>
       <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
+      <c r="J26" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="K26" s="8">
         <v>0.8</v>
       </c>
       <c r="L26" s="8"/>
       <c r="M26" s="8"/>
       <c r="N26" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
@@ -2835,13 +2826,10 @@
         <v>5</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="D27" s="4">
-        <v>0</v>
       </c>
       <c r="E27" s="8">
         <v>4</v>
@@ -2853,14 +2841,16 @@
       <c r="I27" s="8">
         <v>1</v>
       </c>
-      <c r="J27" s="8"/>
+      <c r="J27" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K27" s="8">
         <v>0</v>
       </c>
       <c r="L27" s="8"/>
       <c r="M27" s="8"/>
       <c r="N27" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
@@ -2898,12 +2888,11 @@
         <v>5</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D28" s="4"/>
       <c r="E28" s="8">
         <v>4</v>
       </c>
@@ -2912,14 +2901,16 @@
         <v>1.3</v>
       </c>
       <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
+      <c r="J28" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K28" s="8">
         <v>0</v>
       </c>
       <c r="L28" s="8"/>
       <c r="M28" s="8"/>
       <c r="N28" s="18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
@@ -2957,12 +2948,11 @@
         <v>5</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="4"/>
       <c r="E29" s="8">
         <v>4</v>
       </c>
@@ -2971,14 +2961,16 @@
         <v>1.3</v>
       </c>
       <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
+      <c r="J29" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K29" s="8">
         <v>0</v>
       </c>
       <c r="L29" s="8"/>
       <c r="M29" s="8"/>
       <c r="N29" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
@@ -3016,13 +3008,10 @@
         <v>5</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D30" s="4">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="E30" s="8">
         <v>4</v>
@@ -3032,14 +3021,16 @@
         <v>1.3</v>
       </c>
       <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
+      <c r="J30" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K30" s="8">
         <v>0.3</v>
       </c>
       <c r="L30" s="8"/>
       <c r="M30" s="8"/>
       <c r="N30" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="O30" s="4">
         <v>0.3</v>
@@ -3079,13 +3070,10 @@
         <v>5</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" s="4">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="E31" s="8">
         <v>4</v>
@@ -3095,14 +3083,16 @@
         <v>1.3</v>
       </c>
       <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
+      <c r="J31" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K31" s="8">
         <v>0.7</v>
       </c>
       <c r="L31" s="8"/>
       <c r="M31" s="8"/>
       <c r="N31" s="19" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O31" s="4"/>
       <c r="P31" s="4">
@@ -3146,14 +3136,11 @@
         <v>5</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="4">
-        <v>7</v>
-      </c>
       <c r="E32" s="8">
         <v>2</v>
       </c>
@@ -3164,8 +3151,8 @@
         <v>1.3</v>
       </c>
       <c r="I32" s="8"/>
-      <c r="J32" s="8">
-        <v>3</v>
+      <c r="J32" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="K32" s="8">
         <v>3.7</v>
@@ -3173,7 +3160,7 @@
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
       <c r="N32" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O32" s="4">
         <v>0.4</v>
@@ -3237,14 +3224,11 @@
         <v>5</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D33" s="4">
-        <v>0</v>
-      </c>
       <c r="E33" s="8">
         <v>2</v>
       </c>
@@ -3255,14 +3239,16 @@
         <v>1.2</v>
       </c>
       <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
+      <c r="J33" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K33" s="8">
         <v>0</v>
       </c>
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
       <c r="N33" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
@@ -3300,14 +3286,11 @@
         <v>5</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D34" s="4">
-        <v>0</v>
-      </c>
       <c r="E34" s="8">
         <v>2</v>
       </c>
@@ -3318,14 +3301,16 @@
         <v>1.2</v>
       </c>
       <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
+      <c r="J34" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="K34" s="8">
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
       <c r="M34" s="8"/>
       <c r="N34" s="17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
@@ -3363,14 +3348,11 @@
         <v>5</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D35" s="4">
-        <v>0</v>
-      </c>
       <c r="E35" s="8">
         <v>2</v>
       </c>
@@ -3381,14 +3363,16 @@
         <v>1.2</v>
       </c>
       <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
+      <c r="J35" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="K35" s="8">
         <v>0</v>
       </c>
       <c r="L35" s="8"/>
       <c r="M35" s="8"/>
       <c r="N35" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
@@ -3425,13 +3409,12 @@
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
-      <c r="D36" s="3"/>
       <c r="E36" s="4"/>
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
+      <c r="J36" s="3"/>
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
       <c r="M36" s="8"/>
@@ -3471,13 +3454,12 @@
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
-      <c r="D37" s="3"/>
       <c r="E37" s="4"/>
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
       <c r="H37" s="13"/>
       <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
+      <c r="J37" s="3"/>
       <c r="K37" s="8"/>
       <c r="L37" s="8"/>
       <c r="M37" s="8"/>
@@ -3517,13 +3499,12 @@
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
-      <c r="D38" s="3"/>
       <c r="E38" s="4"/>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
       <c r="H38" s="13"/>
       <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
+      <c r="J38" s="3"/>
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
       <c r="M38" s="8"/>
@@ -3563,13 +3544,12 @@
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
       <c r="C39" s="7"/>
-      <c r="D39" s="3"/>
       <c r="E39" s="4"/>
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
       <c r="H39" s="13"/>
       <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
+      <c r="J39" s="3"/>
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
       <c r="M39" s="8"/>
@@ -3609,13 +3589,12 @@
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
-      <c r="D40" s="3"/>
       <c r="E40" s="4"/>
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
       <c r="H40" s="13"/>
       <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
+      <c r="J40" s="3"/>
       <c r="K40" s="8"/>
       <c r="L40" s="8"/>
       <c r="M40" s="8"/>
@@ -3655,41 +3634,41 @@
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
       <c r="C41" s="8"/>
-      <c r="D41" s="3"/>
       <c r="E41" s="4"/>
       <c r="F41" s="8"/>
       <c r="G41" s="3"/>
       <c r="H41" s="4"/>
+      <c r="J41" s="3"/>
     </row>
     <row r="42" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
       <c r="C42" s="8"/>
-      <c r="D42" s="2"/>
       <c r="E42" s="4"/>
       <c r="F42" s="8"/>
       <c r="G42" s="3"/>
       <c r="H42" s="4"/>
+      <c r="J42" s="2"/>
     </row>
     <row r="43" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="8"/>
-      <c r="D43" s="2"/>
       <c r="E43" s="4"/>
       <c r="F43" s="8"/>
       <c r="G43" s="3"/>
       <c r="H43" s="4"/>
+      <c r="J43" s="2"/>
     </row>
     <row r="44" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="8"/>
-      <c r="D44" s="2"/>
       <c r="E44" s="4"/>
       <c r="F44" s="8"/>
       <c r="G44" s="3"/>
       <c r="H44" s="4"/>
+      <c r="J44" s="2"/>
     </row>
     <row r="45" spans="1:44" x14ac:dyDescent="0.2">
       <c r="C45" s="8"/>

</xml_diff>

<commit_message>
Robust loader: Priority imputation, per-week bruto, unnamed cols dropped, Budget Bucket filtering
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/examples/input_example_realistic_messy.xlsx
+++ b/data/examples/input_example_realistic_messy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/irina.migallon/dev/cli/planzen/data/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46F70AD-EEB7-0740-BE92-746D2729C098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEF30A5-433D-7349-B17A-107CC6DC1EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="680" windowWidth="17300" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="-6460" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="I12" s="8"/>
       <c r="J12" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K12" s="8">
         <v>1.9</v>
@@ -3675,11 +3675,11 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="Y28:Z28"/>
-    <mergeCell ref="Y29:Z29"/>
-    <mergeCell ref="Y30:Z30"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="Y33:Z33"/>
+    <mergeCell ref="Z36:AA36"/>
+    <mergeCell ref="Z38:AA38"/>
+    <mergeCell ref="Z39:AA39"/>
+    <mergeCell ref="Z40:AA40"/>
+    <mergeCell ref="Y35:Z35"/>
     <mergeCell ref="Y34:Z34"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="Z8:AA8"/>
@@ -3690,16 +3690,16 @@
     <mergeCell ref="Y19:Z19"/>
     <mergeCell ref="Y21:Z21"/>
     <mergeCell ref="Y22:Z22"/>
-    <mergeCell ref="Z36:AA36"/>
-    <mergeCell ref="Z38:AA38"/>
-    <mergeCell ref="Z39:AA39"/>
-    <mergeCell ref="Z40:AA40"/>
-    <mergeCell ref="Y35:Z35"/>
     <mergeCell ref="Z23:AA23"/>
     <mergeCell ref="Y24:Z24"/>
     <mergeCell ref="Y26:Z26"/>
     <mergeCell ref="Y27:Z27"/>
     <mergeCell ref="Y16:Z16"/>
+    <mergeCell ref="Y28:Z28"/>
+    <mergeCell ref="Y29:Z29"/>
+    <mergeCell ref="Y30:Z30"/>
+    <mergeCell ref="Y31:Z31"/>
+    <mergeCell ref="Y33:Z33"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N14" r:id="rId1" display="https://tomtom.atlassian.net/browse/NAV-176879" xr:uid="{EC42082B-4739-3742-A30B-AD3EAB48E832}"/>

</xml_diff>